<commit_message>
fix filtros de data infos por periodo em home
</commit_message>
<xml_diff>
--- a/BD/Clientes.xlsx
+++ b/BD/Clientes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Fintracker\BD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{061E2CE7-ADE1-450A-8BC5-985C34A224F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFF82311-9CF9-4815-AF37-D2891A61531D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{12EE3610-CDB3-4D50-AE7B-EBE7A06340D0}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="testeClientes" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="DadosExternos_1" localSheetId="0" hidden="1">testeClientes!$A$1:$L$3</definedName>
+    <definedName name="DadosExternos_1" localSheetId="0" hidden="1">testeClientes!$A$1:$L$9</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="92">
   <si>
     <t>id_Cliente</t>
   </si>
@@ -88,12 +88,6 @@
     <t/>
   </si>
   <si>
-    <t>Ex. Empresa 1</t>
-  </si>
-  <si>
-    <t>Rua Exemplo 123</t>
-  </si>
-  <si>
     <t>Centro</t>
   </si>
   <si>
@@ -103,43 +97,232 @@
     <t>SP</t>
   </si>
   <si>
-    <t>01010-000</t>
-  </si>
-  <si>
-    <t>(11) 91234-5678</t>
-  </si>
-  <si>
-    <t>contato@empresa1.com</t>
-  </si>
-  <si>
     <t>Ativo</t>
   </si>
   <si>
-    <t>Ex. Empresa 2</t>
-  </si>
-  <si>
-    <t>Av. Exemplo 456</t>
-  </si>
-  <si>
-    <t>Jardim</t>
-  </si>
-  <si>
     <t>Rio de Janeiro</t>
   </si>
   <si>
     <t>RJ</t>
   </si>
   <si>
-    <t>22222-222</t>
-  </si>
-  <si>
-    <t>(21) 99876-5432</t>
-  </si>
-  <si>
-    <t>contato@empresa2.com</t>
-  </si>
-  <si>
     <t>Inativo</t>
+  </si>
+  <si>
+    <t>Ex. Empresa 3</t>
+  </si>
+  <si>
+    <t>Rua Alfa 789</t>
+  </si>
+  <si>
+    <t>Bela Vista</t>
+  </si>
+  <si>
+    <t>01310-000</t>
+  </si>
+  <si>
+    <t>20/06/2025 15:30</t>
+  </si>
+  <si>
+    <t>11223344556677</t>
+  </si>
+  <si>
+    <t>(11) 92345-6789</t>
+  </si>
+  <si>
+    <t>contato@empresa3.com</t>
+  </si>
+  <si>
+    <t>Ex. Empresa 4</t>
+  </si>
+  <si>
+    <t>20/06/2025 16:00</t>
+  </si>
+  <si>
+    <t>22334455667788</t>
+  </si>
+  <si>
+    <t>Av. Beta 321</t>
+  </si>
+  <si>
+    <t>Copacabana</t>
+  </si>
+  <si>
+    <t>22040-002</t>
+  </si>
+  <si>
+    <t>(21) 91234-5678</t>
+  </si>
+  <si>
+    <t>contato@empresa4.com</t>
+  </si>
+  <si>
+    <t>Ex. Empresa 5</t>
+  </si>
+  <si>
+    <t>20/06/2025 16:30</t>
+  </si>
+  <si>
+    <t>33445566778899</t>
+  </si>
+  <si>
+    <t>Rua Gamma 654</t>
+  </si>
+  <si>
+    <t>Belo Horizonte</t>
+  </si>
+  <si>
+    <t>MG</t>
+  </si>
+  <si>
+    <t>30140-110</t>
+  </si>
+  <si>
+    <t>(31) 99876-5432</t>
+  </si>
+  <si>
+    <t>contato@empresa5.com</t>
+  </si>
+  <si>
+    <t>Ex. Empresa 6</t>
+  </si>
+  <si>
+    <t>20/06/2025 17:00</t>
+  </si>
+  <si>
+    <t>44556677889900</t>
+  </si>
+  <si>
+    <t>Av. Delta 987</t>
+  </si>
+  <si>
+    <t>Savassi</t>
+  </si>
+  <si>
+    <t>30130-120</t>
+  </si>
+  <si>
+    <t>(31) 98765-4321</t>
+  </si>
+  <si>
+    <t>contato@empresa6.com</t>
+  </si>
+  <si>
+    <t>Ex. Empresa 7</t>
+  </si>
+  <si>
+    <t>20/06/2025 17:30</t>
+  </si>
+  <si>
+    <t>55667788990011</t>
+  </si>
+  <si>
+    <t>Rua Epsilon 111</t>
+  </si>
+  <si>
+    <t>Batel</t>
+  </si>
+  <si>
+    <t>Curitiba</t>
+  </si>
+  <si>
+    <t>PR</t>
+  </si>
+  <si>
+    <t>80420-200</t>
+  </si>
+  <si>
+    <t>(41) 91234-5678</t>
+  </si>
+  <si>
+    <t>contato@empresa7.com</t>
+  </si>
+  <si>
+    <t>Ex. Empresa 8</t>
+  </si>
+  <si>
+    <t>20/06/2025 18:00</t>
+  </si>
+  <si>
+    <t>66778899001122</t>
+  </si>
+  <si>
+    <t>Av. Zeta 222</t>
+  </si>
+  <si>
+    <t>Porto Alegre</t>
+  </si>
+  <si>
+    <t>RS</t>
+  </si>
+  <si>
+    <t>90010-110</t>
+  </si>
+  <si>
+    <t>(51) 99876-5432</t>
+  </si>
+  <si>
+    <t>contato@empresa8.com</t>
+  </si>
+  <si>
+    <t>Ex. Empresa 9</t>
+  </si>
+  <si>
+    <t>20/06/2025 18:30</t>
+  </si>
+  <si>
+    <t>77889900112233</t>
+  </si>
+  <si>
+    <t>Rua Eta 333</t>
+  </si>
+  <si>
+    <t>Boa Viagem</t>
+  </si>
+  <si>
+    <t>Recife</t>
+  </si>
+  <si>
+    <t>PE</t>
+  </si>
+  <si>
+    <t>51020-020</t>
+  </si>
+  <si>
+    <t>(81) 98765-4321</t>
+  </si>
+  <si>
+    <t>contato@empresa9.com</t>
+  </si>
+  <si>
+    <t>Ex. Empresa 10</t>
+  </si>
+  <si>
+    <t>20/06/2025 19:00</t>
+  </si>
+  <si>
+    <t>88990011223344</t>
+  </si>
+  <si>
+    <t>Av. Theta 444</t>
+  </si>
+  <si>
+    <t>Meireles</t>
+  </si>
+  <si>
+    <t>Fortaleza</t>
+  </si>
+  <si>
+    <t>CE</t>
+  </si>
+  <si>
+    <t>60165-121</t>
+  </si>
+  <si>
+    <t>(85) 91234-5678</t>
+  </si>
+  <si>
+    <t>contato@empresa10.com</t>
   </si>
 </sst>
 </file>
@@ -175,11 +358,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -187,13 +371,7 @@
   </cellStyles>
   <dxfs count="12">
     <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ hh:mm"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -215,6 +393,12 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ hh:mm"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -257,20 +441,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1E043718-371C-4A61-A9B4-A90CAE9C7B49}" name="testeClientes" displayName="testeClientes" ref="A1:L3" tableType="queryTable" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1E043718-371C-4A61-A9B4-A90CAE9C7B49}" name="testeClientes" displayName="testeClientes" ref="A1:L9" tableType="queryTable" totalsRowShown="0">
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{E23DB097-A845-4764-B1F8-D8B2E9948120}" uniqueName="1" name="id_Cliente" queryTableFieldId="1" dataDxfId="11"/>
     <tableColumn id="2" xr3:uid="{FAFD4BC7-6374-4192-82E3-FC0A91F65962}" uniqueName="2" name="Nome" queryTableFieldId="2" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{3B88A498-5EB5-4FB7-9077-A8F8C2CEBED1}" uniqueName="3" name="Data_de_Cadastro" queryTableFieldId="3" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{7C2986D8-7C0F-4AF6-AE28-E9639A8E61C2}" uniqueName="4" name="CNPJ" queryTableFieldId="4" dataDxfId="0"/>
-    <tableColumn id="5" xr3:uid="{2AFD315B-B17A-4149-AD01-633DB5AFBF46}" uniqueName="5" name="Endereco" queryTableFieldId="5" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{61ACA624-B77A-49CD-B49C-F2AED98C156A}" uniqueName="6" name="Bairro" queryTableFieldId="6" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{3AC79037-11D0-4CD3-B3AE-F529D05DC096}" uniqueName="7" name="Cidade" queryTableFieldId="7" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{8EDEAD66-4296-4F0A-B16C-54B4C63B7EA9}" uniqueName="8" name="Estado" queryTableFieldId="8" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{E798A977-84EA-442D-9340-2E83A49F5A00}" uniqueName="9" name="CEP" queryTableFieldId="9" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{3DFF8EF5-78B0-434C-B4C7-D2B196693DB5}" uniqueName="10" name="Telefone" queryTableFieldId="10" dataDxfId="5"/>
-    <tableColumn id="11" xr3:uid="{CCEEA646-71C2-4995-A4E2-07701BE6E307}" uniqueName="11" name="Email" queryTableFieldId="11" dataDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{12BBA5AE-1C71-4B92-A8F0-55A818981872}" uniqueName="12" name="Status" queryTableFieldId="12" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{3B88A498-5EB5-4FB7-9077-A8F8C2CEBED1}" uniqueName="3" name="Data_de_Cadastro" queryTableFieldId="3" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{7C2986D8-7C0F-4AF6-AE28-E9639A8E61C2}" uniqueName="4" name="CNPJ" queryTableFieldId="4" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{2AFD315B-B17A-4149-AD01-633DB5AFBF46}" uniqueName="5" name="Endereco" queryTableFieldId="5" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{61ACA624-B77A-49CD-B49C-F2AED98C156A}" uniqueName="6" name="Bairro" queryTableFieldId="6" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{3AC79037-11D0-4CD3-B3AE-F529D05DC096}" uniqueName="7" name="Cidade" queryTableFieldId="7" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{8EDEAD66-4296-4F0A-B16C-54B4C63B7EA9}" uniqueName="8" name="Estado" queryTableFieldId="8" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{E798A977-84EA-442D-9340-2E83A49F5A00}" uniqueName="9" name="CEP" queryTableFieldId="9" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{3DFF8EF5-78B0-434C-B4C7-D2B196693DB5}" uniqueName="10" name="Telefone" queryTableFieldId="10" dataDxfId="2"/>
+    <tableColumn id="11" xr3:uid="{CCEEA646-71C2-4995-A4E2-07701BE6E307}" uniqueName="11" name="Email" queryTableFieldId="11" dataDxfId="1"/>
+    <tableColumn id="12" xr3:uid="{12BBA5AE-1C71-4B92-A8F0-55A818981872}" uniqueName="12" name="Status" queryTableFieldId="12" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -593,12 +777,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{564F5079-C485-4577-BD86-9847300A8B14}">
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="16.7109375" customWidth="1"/>
     <col min="3" max="3" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.140625" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="10" width="16.7109375" customWidth="1"/>
     <col min="11" max="11" width="23" bestFit="1" customWidth="1"/>
     <col min="12" max="13" width="16.7109375" customWidth="1"/>
@@ -614,7 +798,7 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E1" t="s">
@@ -643,83 +827,313 @@
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" s="2">
-        <v>45828.604166666664</v>
-      </c>
-      <c r="D2" s="3">
-        <v>12345678000199</v>
-      </c>
-      <c r="E2" s="1" t="s">
+      <c r="B2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="H2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="I2" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="L2" s="3" t="s">
         <v>16</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" s="2">
-        <v>45828.625</v>
-      </c>
-      <c r="D3" s="3">
-        <v>98765432000188</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J3" s="1" t="s">
+      <c r="B3" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="L3" s="1" t="s">
+      <c r="D3" s="2" t="s">
         <v>30</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" s="3"/>
+      <c r="B6" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" s="3"/>
+      <c r="B7" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="J8" s="4"/>
+      <c r="A8" s="3"/>
+      <c r="B8" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" s="3"/>
+      <c r="B9" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" s="4"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
+      <c r="K10" s="4"/>
+      <c r="L10" s="4"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C13" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>